<commit_message>
Rework task lifecycle: Start/Complete/Abandoned, adaptive duration, Defer replaces enabled/unavailable/never-suggest
</commit_message>
<xml_diff>
--- a/content/microtasking-sheet-template.xlsx
+++ b/content/microtasking-sheet-template.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,11 +429,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>durationMinutes</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>link</t>
         </is>
       </c>
@@ -444,10 +439,6 @@
           <t>Find 3 things you don't need and throw them away.</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -455,10 +446,6 @@
           <t>Clear off one flat surface completely (desk, counter, nightstand).</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -466,10 +453,6 @@
           <t>Empty one trash/recycling bin that isn't empty yet.</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -477,10 +460,6 @@
           <t>Sort the mail pile into keep / recycle / shred.</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -488,10 +467,6 @@
           <t>Put away 5 items that are out of place.</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -499,10 +474,6 @@
           <t>Empty your bag or pockets and toss any trash/receipts inside.</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -510,10 +481,6 @@
           <t>Clear expired or unused items off one shelf.</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -521,10 +488,6 @@
           <t>Delete 10 apps or photos you don't need from your phone.</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>5</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -532,10 +495,6 @@
           <t>Toss expired food from the fridge door or one shelf.</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -543,10 +502,6 @@
           <t>Gather stray cords/cables into a pile and toss the broken ones.</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -554,10 +509,6 @@
           <t>Clear out one kitchen drawer.</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -565,10 +516,6 @@
           <t>Sort through the stack of papers on your desk.</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>10</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -576,10 +523,6 @@
           <t>Go through your closet and pull 5 items to donate.</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -587,10 +530,6 @@
           <t>Wipe down and organize one bathroom cabinet or drawer.</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>10</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -598,10 +537,6 @@
           <t>Consolidate duplicate pantry items (spices, condiments, etc.).</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>10</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -609,10 +544,6 @@
           <t>Sort your sock/underwear drawer; pair or toss the unmatched ones.</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>10</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -620,10 +551,6 @@
           <t>Clear off and reorganize one bookshelf.</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>10</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -631,10 +558,6 @@
           <t>Go through your car's glovebox and center console.</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>10</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -642,10 +565,6 @@
           <t>Sort through "the junk drawer."</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>10</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -653,10 +572,6 @@
           <t>Organize shoes by the front door; remove pairs you don't wear.</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>10</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -664,10 +579,6 @@
           <t>Clean out one section of your closet and bag up donations.</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>15</v>
-      </c>
-      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -675,10 +586,6 @@
           <t>Go through a box you haven't opened in months.</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>15</v>
-      </c>
-      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -686,10 +593,6 @@
           <t>Fully declutter your desktop workspace — cables, papers, supplies.</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>15</v>
-      </c>
-      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -697,10 +600,6 @@
           <t>Sort through your bathroom counter/cabinet and toss old products.</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>15</v>
-      </c>
-      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -708,10 +607,6 @@
           <t>Go through your bookshelf and box up books to donate.</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>15</v>
-      </c>
-      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -719,10 +614,6 @@
           <t>Clear out the top of the fridge or a high cabinet you avoid.</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>15</v>
-      </c>
-      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -730,10 +621,6 @@
           <t>Sort the linen closet — towels/sheets you don't use.</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>15</v>
-      </c>
-      <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -741,10 +628,6 @@
           <t>Go through the garage or entryway and remove items that don't belong there.</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>15</v>
-      </c>
-      <c r="C29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -757,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -768,11 +651,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>durationMinutes</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>link</t>
         </is>
       </c>
@@ -783,10 +661,6 @@
           <t>Wipe down the kitchen counters.</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -794,10 +668,6 @@
           <t>Wipe down the bathroom sink and faucet.</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -805,10 +675,6 @@
           <t>Spot-clean one mirror or window.</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -816,10 +682,6 @@
           <t>Wipe down the stovetop.</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -827,10 +689,6 @@
           <t>Quick sweep of one room's floor.</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -838,10 +696,6 @@
           <t>Wipe down light switches and door handles.</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -849,10 +703,6 @@
           <t>Rinse the dishes sitting in the sink.</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -860,10 +710,6 @@
           <t>Wipe down the microwave inside and out.</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>5</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -871,10 +717,6 @@
           <t>Vacuum one room.</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -882,10 +724,6 @@
           <t>Clean the toilet.</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -893,10 +731,6 @@
           <t>Wipe down kitchen appliance exteriors (fridge, toaster, etc.).</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -904,10 +738,6 @@
           <t>Sweep and mop one small floor area (kitchen/bathroom).</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>10</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -915,10 +745,6 @@
           <t>Dust one room's surfaces (shelves, tables).</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -926,10 +752,6 @@
           <t>Clean the shower or tub.</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>10</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -937,10 +759,6 @@
           <t>Wipe down baseboards in one room.</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>10</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -948,10 +766,6 @@
           <t>Deep-wipe the inside of the microwave, including the turntable.</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>10</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -959,10 +773,6 @@
           <t>Vacuum and mop an entire room.</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -970,10 +780,6 @@
           <t>Deep clean the bathroom (toilet, sink, tub, mirror).</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -981,10 +787,6 @@
           <t>Clean the inside of the refrigerator.</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>15</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -992,10 +794,6 @@
           <t>Wash a full sink of dishes.</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>15</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1003,10 +801,6 @@
           <t>Clean the windows in one room, inside and out.</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>15</v>
-      </c>
-      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1014,10 +808,6 @@
           <t>Dust and wipe down all furniture in one room.</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>15</v>
-      </c>
-      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1025,10 +815,6 @@
           <t>Clean out and wipe down the oven interior (surface level).</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>15</v>
-      </c>
-      <c r="C24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1041,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1052,11 +838,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>durationMinutes</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>link</t>
         </is>
       </c>
@@ -1067,10 +848,6 @@
           <t>Open and sort today's mail.</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1078,10 +855,6 @@
           <t>Shred one pile of old documents.</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1089,10 +862,6 @@
           <t>File one document that's been sitting out.</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1100,10 +869,6 @@
           <t>Update one contact's info in your phone.</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1111,10 +876,6 @@
           <t>Set a reminder for one upcoming due date or bill.</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1122,10 +883,6 @@
           <t>Unsubscribe from 3 unwanted emails or newsletters.</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1133,10 +890,6 @@
           <t>Scan or photograph one important document for your records.</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1144,10 +897,6 @@
           <t>Pay one outstanding bill.</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1155,10 +904,6 @@
           <t>Sort through a stack of paperwork into keep/file/shred.</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1166,10 +911,6 @@
           <t>Renew or schedule renewal of one subscription, license, or registration.</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1177,10 +918,6 @@
           <t>Fill out one pending form.</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1188,10 +925,6 @@
           <t>Update your calendar with upcoming appointments or deadlines.</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>10</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1199,10 +932,6 @@
           <t>Organize digital files on your desktop into folders.</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1210,10 +939,6 @@
           <t>Review and respond to one important email you've been avoiding.</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>10</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1221,10 +946,6 @@
           <t>Set up autopay or reminders for a recurring bill.</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1232,10 +953,6 @@
           <t>Organize a full folder or drawer of physical documents.</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1243,10 +960,6 @@
           <t>Review your subscriptions and cancel the ones you don't use.</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1254,10 +967,6 @@
           <t>Complete one section of a longer form (taxes, insurance, etc.).</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1265,10 +974,6 @@
           <t>Back up your important files or photos.</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>15</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1276,10 +981,6 @@
           <t>Draft and send one email you've been putting off.</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>15</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1292,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1303,11 +1004,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>durationMinutes</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>link</t>
         </is>
       </c>
@@ -1318,10 +1014,6 @@
           <t>Check your bank account balance and recent transactions.</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1329,10 +1021,6 @@
           <t>Log one recent expense in your budget or app.</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1340,10 +1028,6 @@
           <t>Move a small amount into savings.</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1351,10 +1035,6 @@
           <t>Check for any unexpected charges on your statement.</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1362,10 +1042,6 @@
           <t>Review one upcoming bill's due date.</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1373,10 +1049,6 @@
           <t>Round up loose cash or coins and put them into savings.</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1384,10 +1056,6 @@
           <t>Categorize last week's transactions in your budgeting app.</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>10</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1395,10 +1063,6 @@
           <t>Compare prices on one recurring expense (insurance, phone plan, etc.).</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1406,10 +1070,6 @@
           <t>Review your credit card statement for errors.</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1417,10 +1077,6 @@
           <t>Set or adjust a budget for one spending category.</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1428,10 +1084,6 @@
           <t>Check your credit score.</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1439,10 +1091,6 @@
           <t>Cancel one unused subscription or service.</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>10</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1450,10 +1098,6 @@
           <t>Reconcile your budget for the week or month.</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>15</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1461,10 +1105,6 @@
           <t>Research and compare rates for one bill (insurance, utilities).</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1472,10 +1112,6 @@
           <t>Review your retirement or investment account balances.</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1483,10 +1119,6 @@
           <t>Set up or adjust automatic transfers to savings or investments.</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1494,10 +1126,6 @@
           <t>Create or update a simple monthly budget.</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1505,10 +1133,6 @@
           <t>Review your net worth (assets minus debts).</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1521,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1532,11 +1156,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>durationMinutes</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>link</t>
         </is>
       </c>
@@ -1547,10 +1166,6 @@
           <t>Take today's medication or vitamins.</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1558,10 +1173,6 @@
           <t>Schedule a doctor or dentist appointment you've been putting off.</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1569,10 +1180,6 @@
           <t>Refill one prescription.</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1580,10 +1187,6 @@
           <t>Do a quick stretch routine.</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1591,10 +1194,6 @@
           <t>Drink a full glass of water and refill your water bottle.</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1602,10 +1201,6 @@
           <t>Log today's meals or water in a health app.</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1613,10 +1208,6 @@
           <t>Do 20 pushups/squats or a short burst of exercise.</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1624,10 +1215,6 @@
           <t>Go for a short walk.</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1635,10 +1222,6 @@
           <t>Do a full stretching routine.</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1646,10 +1229,6 @@
           <t>Prep a healthy snack or meal for tomorrow.</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1657,10 +1236,6 @@
           <t>Call to confirm or reschedule an upcoming appointment.</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1668,10 +1243,6 @@
           <t>Do a quick home workout video.</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>10</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1679,10 +1250,6 @@
           <t>Organize your medicine cabinet and check expiration dates.</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1690,10 +1257,6 @@
           <t>Go for a brisk walk or short jog.</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1701,10 +1264,6 @@
           <t>Do a full home workout session.</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1712,10 +1271,6 @@
           <t>Meal-prep one healthy dish for the week.</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1723,10 +1278,6 @@
           <t>Research and book a needed medical or dental appointment.</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1734,10 +1285,6 @@
           <t>Organize your health records or insurance documents.</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1750,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1761,11 +1308,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>durationMinutes</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>link</t>
         </is>
       </c>
@@ -1776,10 +1318,6 @@
           <t>Add missing items to your grocery list.</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1787,10 +1325,6 @@
           <t>Take out the trash/recycling.</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1798,10 +1332,6 @@
           <t>Start the errand of putting gas in the car if it's low.</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1809,10 +1339,6 @@
           <t>Gather items that need to be returned to a store.</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1820,10 +1346,6 @@
           <t>Water your plants.</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1831,10 +1353,6 @@
           <t>Bring in the mail or packages.</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1842,10 +1360,6 @@
           <t>Set aside a bag of items to donate or drop off.</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1853,10 +1367,6 @@
           <t>Pack a return package and prepare the shipping label.</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1864,10 +1374,6 @@
           <t>Drop off or pick up dry cleaning.</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1875,10 +1381,6 @@
           <t>Wash the car (quick exterior rinse).</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1886,10 +1388,6 @@
           <t>Take pets for a quick walk, feed them, and refill supplies.</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1897,10 +1395,6 @@
           <t>Organize your car — remove trash, wipe down surfaces.</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>10</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1908,10 +1402,6 @@
           <t>Prepare a grocery list and meal plan for the week.</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1919,10 +1409,6 @@
           <t>Do a full grocery run for a few essential items.</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1930,10 +1416,6 @@
           <t>Take a bag of donations to a donation center.</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1941,10 +1423,6 @@
           <t>Wash and detail the interior of your car.</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1952,10 +1430,6 @@
           <t>Run multiple small errands in one trip (post office, pharmacy, store).</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1963,10 +1437,6 @@
           <t>Take pets to a grooming or vet appointment.</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update sheet template script to 3-column format (checkbox, description, link)
</commit_message>
<xml_diff>
--- a/content/microtasking-sheet-template.xlsx
+++ b/content/microtasking-sheet-template.xlsx
@@ -418,212 +418,301 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Find 3 things you don't need and throw them away.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Clear off one flat surface completely (desk, counter, nightstand).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Empty one trash/recycling bin that isn't empty yet.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Sort the mail pile into keep / recycle / shred.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Put away 5 items that are out of place.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Empty your bag or pockets and toss any trash/receipts inside.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Clear expired or unused items off one shelf.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Delete 10 apps or photos you don't need from your phone.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Toss expired food from the fridge door or one shelf.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Gather stray cords/cables into a pile and toss the broken ones.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Clear out one kitchen drawer.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Sort through the stack of papers on your desk.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Go through your closet and pull 5 items to donate.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Wipe down and organize one bathroom cabinet or drawer.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Consolidate duplicate pantry items (spices, condiments, etc.).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Sort your sock/underwear drawer; pair or toss the unmatched ones.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Clear off and reorganize one bookshelf.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Go through your car's glovebox and center console.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Sort through "the junk drawer."</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Organize shoes by the front door; remove pairs you don't wear.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>Clean out one section of your closet and bag up donations.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Go through a box you haven't opened in months.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Fully declutter your desktop workspace — cables, papers, supplies.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>Sort through your bathroom counter/cabinet and toss old products.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" t="b">
+        <v>1</v>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Go through your bookshelf and box up books to donate.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" t="b">
+        <v>1</v>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>Clear out the top of the fridge or a high cabinet you avoid.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" t="b">
+        <v>1</v>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>Sort the linen closet — towels/sheets you don't use.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" t="b">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>Go through the garage or entryway and remove items that don't belong there.</t>
         </is>
@@ -640,177 +729,251 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Wipe down the kitchen counters.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Wipe down the bathroom sink and faucet.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Spot-clean one mirror or window.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Wipe down the stovetop.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Quick sweep of one room's floor.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Wipe down light switches and door handles.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Rinse the dishes sitting in the sink.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Wipe down the microwave inside and out.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Vacuum one room.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Clean the toilet.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Wipe down kitchen appliance exteriors (fridge, toaster, etc.).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Sweep and mop one small floor area (kitchen/bathroom).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Dust one room's surfaces (shelves, tables).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Clean the shower or tub.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Wipe down baseboards in one room.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Deep-wipe the inside of the microwave, including the turntable.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Vacuum and mop an entire room.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Deep clean the bathroom (toilet, sink, tub, mirror).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Clean the inside of the refrigerator.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Wash a full sink of dishes.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>Clean the windows in one room, inside and out.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Dust and wipe down all furniture in one room.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Clean out and wipe down the oven interior (surface level).</t>
         </is>
@@ -827,156 +990,221 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Open and sort today's mail.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Shred one pile of old documents.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>File one document that's been sitting out.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Update one contact's info in your phone.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Set a reminder for one upcoming due date or bill.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Unsubscribe from 3 unwanted emails or newsletters.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Scan or photograph one important document for your records.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Pay one outstanding bill.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Sort through a stack of paperwork into keep/file/shred.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Renew or schedule renewal of one subscription, license, or registration.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Fill out one pending form.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Update your calendar with upcoming appointments or deadlines.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Organize digital files on your desktop into folders.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Review and respond to one important email you've been avoiding.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Set up autopay or reminders for a recurring bill.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Organize a full folder or drawer of physical documents.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Review your subscriptions and cancel the ones you don't use.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Complete one section of a longer form (taxes, insurance, etc.).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Back up your important files or photos.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Draft and send one email you've been putting off.</t>
         </is>
@@ -993,142 +1221,201 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Check your bank account balance and recent transactions.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Log one recent expense in your budget or app.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Move a small amount into savings.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Check for any unexpected charges on your statement.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Review one upcoming bill's due date.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Round up loose cash or coins and put them into savings.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Categorize last week's transactions in your budgeting app.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Compare prices on one recurring expense (insurance, phone plan, etc.).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Review your credit card statement for errors.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Set or adjust a budget for one spending category.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Check your credit score.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Cancel one unused subscription or service.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Reconcile your budget for the week or month.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Research and compare rates for one bill (insurance, utilities).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Review your retirement or investment account balances.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Set up or adjust automatic transfers to savings or investments.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Create or update a simple monthly budget.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Review your net worth (assets minus debts).</t>
         </is>
@@ -1145,142 +1432,201 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Take today's medication or vitamins.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Schedule a doctor or dentist appointment you've been putting off.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Refill one prescription.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Do a quick stretch routine.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Drink a full glass of water and refill your water bottle.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Log today's meals or water in a health app.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Do 20 pushups/squats or a short burst of exercise.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Go for a short walk.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Do a full stretching routine.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Prep a healthy snack or meal for tomorrow.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Call to confirm or reschedule an upcoming appointment.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Do a quick home workout video.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Organize your medicine cabinet and check expiration dates.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Go for a brisk walk or short jog.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Do a full home workout session.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Meal-prep one healthy dish for the week.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Research and book a needed medical or dental appointment.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Organize your health records or insurance documents.</t>
         </is>
@@ -1297,142 +1643,201 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Add missing items to your grocery list.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Take out the trash/recycling.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Start the errand of putting gas in the car if it's low.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Gather items that need to be returned to a store.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Water your plants.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Bring in the mail or packages.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Set aside a bag of items to donate or drop off.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Pack a return package and prepare the shipping label.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Drop off or pick up dry cleaning.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Wash the car (quick exterior rinse).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Take pets for a quick walk, feed them, and refill supplies.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Organize your car — remove trash, wipe down surfaces.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Prepare a grocery list and meal plan for the week.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Do a full grocery run for a few essential items.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Take a bag of donations to a donation center.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Wash and detail the interior of your car.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Run multiple small errands in one trip (post office, pharmacy, store).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Take pets to a grooming or vet appointment.</t>
         </is>

</xml_diff>

<commit_message>
Add Google Apps Script and update Excel template for 3-column format with master toggle and README
</commit_message>
<xml_diff>
--- a/content/microtasking-sheet-template.xlsx
+++ b/content/microtasking-sheet-template.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Decluttering" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cleaning" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Admin - Paperwork" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Finances" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Health" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Errands" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Decluttering" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cleaning" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Paperwork" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Finances" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Health" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Errands" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,303 +419,119 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>link</t>
+          <t>MICROTASKING TASK POOL TEMPLATE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Find 3 things you don't need and throw them away.</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="b">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Clear off one flat surface completely (desk, counter, nightstand).</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Welcome to your MicroTasking Task Pool spreadsheet!</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="b">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Empty one trash/recycling bin that isn't empty yet.</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="b">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Sort the mail pile into keep / recycle / shred.</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HOW TO USE THIS SPREADSHEET:</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="b">
-        <v>1</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Put away 5 items that are out of place.</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1. CATEGORIES (TABS): Each tab at the bottom represents a category (e.g. Decluttering, Cleaning, Paperwork, Finances, Health, Errands).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Empty your bag or pockets and toss any trash/receipts inside.</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - You can add new tabs, rename existing tabs, or delete tabs you don't need.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
-        <v>1</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Clear expired or unused items off one shelf.</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Delete 10 apps or photos you don't need from your phone.</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2. COLUMNS IN TASK TABS:</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Toss expired food from the fridge door or one shelf.</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Column A (Row 1 Master Toggle / Checkbox): Cell A1 controls all checkboxes in Column A below it.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Gather stray cords/cables into a pile and toss the broken ones.</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Check A1 to enable all tasks in the category, or uncheck A1 to disable all tasks.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Clear out one kitchen drawer.</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Column B (Description): The text description of the micro-task.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
-        <v>1</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Sort through the stack of papers on your desk.</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Column C (Link): Optional URL (e.g. video tutorial, document, or web tool).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Go through your closet and pull 5 items to donate.</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Wipe down and organize one bathroom cabinet or drawer.</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3. SYNCING WITH THE APP:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Consolidate duplicate pantry items (spices, condiments, etc.).</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Set Share permissions to 'Anyone with the link can view'.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Sort your sock/underwear drawer; pair or toss the unmatched ones.</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Paste your Sheet URL into the onboarding page to generate your custom QR code.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="b">
-        <v>1</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Clear off and reorganize one bookshelf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="b">
-        <v>1</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Go through your car's glovebox and center console.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="b">
-        <v>1</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Sort through "the junk drawer."</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="b">
-        <v>1</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Organize shoes by the front door; remove pairs you don't wear.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="b">
-        <v>1</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Clean out one section of your closet and bag up donations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Go through a box you haven't opened in months.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="b">
-        <v>1</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Fully declutter your desktop workspace — cables, papers, supplies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Sort through your bathroom counter/cabinet and toss old products.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="b">
-        <v>1</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Go through your bookshelf and box up books to donate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="b">
-        <v>1</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Clear out the top of the fridge or a high cabinet you avoid.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="b">
-        <v>1</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Sort the linen closet — towels/sheets you don't use.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="b">
-        <v>1</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Go through the garage or entryway and remove items that don't belong there.</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - In the MicroTasking app, tap Settings -&gt; Import External Task Pool -&gt; Scan QR Code.</t>
         </is>
       </c>
     </row>
@@ -729,14 +546,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
+      <c r="A1" t="b">
+        <v>1</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>
@@ -750,232 +570,310 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="b">
-        <v>1</v>
+      <c r="A2">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Wipe down the kitchen counters.</t>
+          <t>Find 3 things you don't need and throw them away.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="b">
-        <v>1</v>
+      <c r="A3">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wipe down the bathroom sink and faucet.</t>
+          <t>Clear off one flat surface completely (desk, counter, nightstand).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="b">
-        <v>1</v>
+      <c r="A4">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Spot-clean one mirror or window.</t>
+          <t>Empty one trash/recycling bin that isn't empty yet.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="b">
-        <v>1</v>
+      <c r="A5">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Wipe down the stovetop.</t>
+          <t>Sort the mail pile into keep / recycle / shred.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="b">
-        <v>1</v>
+      <c r="A6">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Quick sweep of one room's floor.</t>
+          <t>Put away 5 items that are out of place.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
-        <v>1</v>
+      <c r="A7">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wipe down light switches and door handles.</t>
+          <t>Empty your bag or pockets and toss any trash/receipts inside.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
-        <v>1</v>
+      <c r="A8">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rinse the dishes sitting in the sink.</t>
+          <t>Clear expired or unused items off one shelf.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="b">
-        <v>1</v>
+      <c r="A9">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wipe down the microwave inside and out.</t>
+          <t>Delete 10 apps or photos you don't need from your phone.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
-        <v>1</v>
+      <c r="A10">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Vacuum one room.</t>
+          <t>Toss expired food from the fridge door or one shelf.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
-        <v>1</v>
+      <c r="A11">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Clean the toilet.</t>
+          <t>Gather stray cords/cables into a pile and toss the broken ones.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
-        <v>1</v>
+      <c r="A12">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Wipe down kitchen appliance exteriors (fridge, toaster, etc.).</t>
+          <t>Clear out one kitchen drawer.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
-        <v>1</v>
+      <c r="A13">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sweep and mop one small floor area (kitchen/bathroom).</t>
+          <t>Sort through the stack of papers on your desk.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
-        <v>1</v>
+      <c r="A14">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dust one room's surfaces (shelves, tables).</t>
+          <t>Go through your closet and pull 5 items to donate.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
+      <c r="A15">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Clean the shower or tub.</t>
+          <t>Wipe down and organize one bathroom cabinet or drawer.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
+      <c r="A16">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wipe down baseboards in one room.</t>
+          <t>Consolidate duplicate pantry items (spices, condiments, etc.).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="b">
-        <v>1</v>
+      <c r="A17">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Deep-wipe the inside of the microwave, including the turntable.</t>
+          <t>Sort your sock/underwear drawer; pair or toss the unmatched ones.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="b">
-        <v>1</v>
+      <c r="A18">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Vacuum and mop an entire room.</t>
+          <t>Clear off and reorganize one bookshelf.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="b">
-        <v>1</v>
+      <c r="A19">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deep clean the bathroom (toilet, sink, tub, mirror).</t>
+          <t>Go through your car's glovebox and center console.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="b">
-        <v>1</v>
+      <c r="A20">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Clean the inside of the refrigerator.</t>
+          <t>Sort through "the junk drawer."</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="b">
-        <v>1</v>
+      <c r="A21">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Wash a full sink of dishes.</t>
+          <t>Organize shoes by the front door; remove pairs you don't wear.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="b">
-        <v>1</v>
+      <c r="A22">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Clean the windows in one room, inside and out.</t>
+          <t>Clean out one section of your closet and bag up donations.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="b">
-        <v>1</v>
+      <c r="A23">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dust and wipe down all furniture in one room.</t>
+          <t>Go through a box you haven't opened in months.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="b">
-        <v>1</v>
+      <c r="A24">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Clean out and wipe down the oven interior (surface level).</t>
+          <t>Fully declutter your desktop workspace — cables, papers, supplies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sort through your bathroom counter/cabinet and toss old products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Go through your bookshelf and box up books to donate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Clear out the top of the fridge or a high cabinet you avoid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Sort the linen closet — towels/sheets you don't use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Go through the garage or entryway and remove items that don't belong there.</t>
         </is>
       </c>
     </row>
@@ -990,14 +888,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
+      <c r="A1" t="b">
+        <v>1</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>
@@ -1011,202 +912,255 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="b">
-        <v>1</v>
+      <c r="A2">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open and sort today's mail.</t>
+          <t>Wipe down the kitchen counters.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="b">
-        <v>1</v>
+      <c r="A3">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Shred one pile of old documents.</t>
+          <t>Wipe down the bathroom sink and faucet.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="b">
-        <v>1</v>
+      <c r="A4">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>File one document that's been sitting out.</t>
+          <t>Spot-clean one mirror or window.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="b">
-        <v>1</v>
+      <c r="A5">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Update one contact's info in your phone.</t>
+          <t>Wipe down the stovetop.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="b">
-        <v>1</v>
+      <c r="A6">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Set a reminder for one upcoming due date or bill.</t>
+          <t>Quick sweep of one room's floor.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
-        <v>1</v>
+      <c r="A7">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Unsubscribe from 3 unwanted emails or newsletters.</t>
+          <t>Wipe down light switches and door handles.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
-        <v>1</v>
+      <c r="A8">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Scan or photograph one important document for your records.</t>
+          <t>Rinse the dishes sitting in the sink.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="b">
-        <v>1</v>
+      <c r="A9">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pay one outstanding bill.</t>
+          <t>Wipe down the microwave inside and out.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
-        <v>1</v>
+      <c r="A10">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sort through a stack of paperwork into keep/file/shred.</t>
+          <t>Vacuum one room.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
-        <v>1</v>
+      <c r="A11">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Renew or schedule renewal of one subscription, license, or registration.</t>
+          <t>Clean the toilet.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
-        <v>1</v>
+      <c r="A12">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fill out one pending form.</t>
+          <t>Wipe down kitchen appliance exteriors (fridge, toaster, etc.).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
-        <v>1</v>
+      <c r="A13">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Update your calendar with upcoming appointments or deadlines.</t>
+          <t>Sweep and mop one small floor area (kitchen/bathroom).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
-        <v>1</v>
+      <c r="A14">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Organize digital files on your desktop into folders.</t>
+          <t>Dust one room's surfaces (shelves, tables).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
+      <c r="A15">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Review and respond to one important email you've been avoiding.</t>
+          <t>Clean the shower or tub.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
+      <c r="A16">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Set up autopay or reminders for a recurring bill.</t>
+          <t>Wipe down baseboards in one room.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="b">
-        <v>1</v>
+      <c r="A17">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Organize a full folder or drawer of physical documents.</t>
+          <t>Deep-wipe the inside of the microwave, including the turntable.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="b">
-        <v>1</v>
+      <c r="A18">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Review your subscriptions and cancel the ones you don't use.</t>
+          <t>Vacuum and mop an entire room.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="b">
-        <v>1</v>
+      <c r="A19">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Complete one section of a longer form (taxes, insurance, etc.).</t>
+          <t>Deep clean the bathroom (toilet, sink, tub, mirror).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="b">
-        <v>1</v>
+      <c r="A20">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Back up your important files or photos.</t>
+          <t>Clean the inside of the refrigerator.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="b">
-        <v>1</v>
+      <c r="A21">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Draft and send one email you've been putting off.</t>
+          <t>Wash a full sink of dishes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Clean the windows in one room, inside and out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Dust and wipe down all furniture in one room.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Clean out and wipe down the oven interior (surface level).</t>
         </is>
       </c>
     </row>
@@ -1221,14 +1175,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
+      <c r="A1" t="b">
+        <v>1</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>
@@ -1242,182 +1199,222 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="b">
-        <v>1</v>
+      <c r="A2">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Check your bank account balance and recent transactions.</t>
+          <t>Open and sort today's mail.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="b">
-        <v>1</v>
+      <c r="A3">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Log one recent expense in your budget or app.</t>
+          <t>Shred one pile of old documents.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="b">
-        <v>1</v>
+      <c r="A4">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Move a small amount into savings.</t>
+          <t>File one document that's been sitting out.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="b">
-        <v>1</v>
+      <c r="A5">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Check for any unexpected charges on your statement.</t>
+          <t>Update one contact's info in your phone.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="b">
-        <v>1</v>
+      <c r="A6">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Review one upcoming bill's due date.</t>
+          <t>Set a reminder for one upcoming due date or bill.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
-        <v>1</v>
+      <c r="A7">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Round up loose cash or coins and put them into savings.</t>
+          <t>Unsubscribe from 3 unwanted emails or newsletters.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
-        <v>1</v>
+      <c r="A8">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Categorize last week's transactions in your budgeting app.</t>
+          <t>Scan or photograph one important document for your records.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="b">
-        <v>1</v>
+      <c r="A9">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Compare prices on one recurring expense (insurance, phone plan, etc.).</t>
+          <t>Pay one outstanding bill.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
-        <v>1</v>
+      <c r="A10">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Review your credit card statement for errors.</t>
+          <t>Sort through a stack of paperwork into keep/file/shred.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
-        <v>1</v>
+      <c r="A11">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Set or adjust a budget for one spending category.</t>
+          <t>Renew or schedule renewal of one subscription, license, or registration.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
-        <v>1</v>
+      <c r="A12">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Check your credit score.</t>
+          <t>Fill out one pending form.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
-        <v>1</v>
+      <c r="A13">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cancel one unused subscription or service.</t>
+          <t>Update your calendar with upcoming appointments or deadlines.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
-        <v>1</v>
+      <c r="A14">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Reconcile your budget for the week or month.</t>
+          <t>Organize digital files on your desktop into folders.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
+      <c r="A15">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Research and compare rates for one bill (insurance, utilities).</t>
+          <t>Review and respond to one important email you've been avoiding.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
+      <c r="A16">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Review your retirement or investment account balances.</t>
+          <t>Set up autopay or reminders for a recurring bill.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="b">
-        <v>1</v>
+      <c r="A17">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Set up or adjust automatic transfers to savings or investments.</t>
+          <t>Organize a full folder or drawer of physical documents.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="b">
-        <v>1</v>
+      <c r="A18">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Create or update a simple monthly budget.</t>
+          <t>Review your subscriptions and cancel the ones you don't use.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="b">
-        <v>1</v>
+      <c r="A19">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Review your net worth (assets minus debts).</t>
+          <t>Complete one section of a longer form (taxes, insurance, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Back up your important files or photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Draft and send one email you've been putting off.</t>
         </is>
       </c>
     </row>
@@ -1434,12 +1431,15 @@
   </sheetPr>
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
+      <c r="A1" t="b">
+        <v>1</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>
@@ -1453,182 +1453,200 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="b">
-        <v>1</v>
+      <c r="A2">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Take today's medication or vitamins.</t>
+          <t>Check your bank account balance and recent transactions.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="b">
-        <v>1</v>
+      <c r="A3">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Schedule a doctor or dentist appointment you've been putting off.</t>
+          <t>Log one recent expense in your budget or app.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="b">
-        <v>1</v>
+      <c r="A4">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Refill one prescription.</t>
+          <t>Move a small amount into savings.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="b">
-        <v>1</v>
+      <c r="A5">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Do a quick stretch routine.</t>
+          <t>Check for any unexpected charges on your statement.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="b">
-        <v>1</v>
+      <c r="A6">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Drink a full glass of water and refill your water bottle.</t>
+          <t>Review one upcoming bill's due date.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
-        <v>1</v>
+      <c r="A7">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Log today's meals or water in a health app.</t>
+          <t>Round up loose cash or coins and put them into savings.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
-        <v>1</v>
+      <c r="A8">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Do 20 pushups/squats or a short burst of exercise.</t>
+          <t>Categorize last week's transactions in your budgeting app.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="b">
-        <v>1</v>
+      <c r="A9">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Go for a short walk.</t>
+          <t>Compare prices on one recurring expense (insurance, phone plan, etc.).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
-        <v>1</v>
+      <c r="A10">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Do a full stretching routine.</t>
+          <t>Review your credit card statement for errors.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
-        <v>1</v>
+      <c r="A11">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prep a healthy snack or meal for tomorrow.</t>
+          <t>Set or adjust a budget for one spending category.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
-        <v>1</v>
+      <c r="A12">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Call to confirm or reschedule an upcoming appointment.</t>
+          <t>Check your credit score.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
-        <v>1</v>
+      <c r="A13">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Do a quick home workout video.</t>
+          <t>Cancel one unused subscription or service.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
-        <v>1</v>
+      <c r="A14">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Organize your medicine cabinet and check expiration dates.</t>
+          <t>Reconcile your budget for the week or month.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
+      <c r="A15">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Go for a brisk walk or short jog.</t>
+          <t>Research and compare rates for one bill (insurance, utilities).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
+      <c r="A16">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Do a full home workout session.</t>
+          <t>Review your retirement or investment account balances.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="b">
-        <v>1</v>
+      <c r="A17">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Meal-prep one healthy dish for the week.</t>
+          <t>Set up or adjust automatic transfers to savings or investments.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="b">
-        <v>1</v>
+      <c r="A18">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Research and book a needed medical or dental appointment.</t>
+          <t>Create or update a simple monthly budget.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="b">
-        <v>1</v>
+      <c r="A19">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Organize your health records or insurance documents.</t>
+          <t>Review your net worth (assets minus debts).</t>
         </is>
       </c>
     </row>
@@ -1645,12 +1663,15 @@
   </sheetPr>
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
+      <c r="A1" t="b">
+        <v>1</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>
@@ -1664,9 +1685,242 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="b">
+      <c r="A2">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Take today's medication or vitamins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Schedule a doctor or dentist appointment you've been putting off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Refill one prescription.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Do a quick stretch routine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Drink a full glass of water and refill your water bottle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Log today's meals or water in a health app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Do 20 pushups/squats or a short burst of exercise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Go for a short walk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Do a full stretching routine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Prep a healthy snack or meal for tomorrow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Call to confirm or reschedule an upcoming appointment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Do a quick home workout video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Organize your medicine cabinet and check expiration dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Go for a brisk walk or short jog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Do a full home workout session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Meal-prep one healthy dish for the week.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Research and book a needed medical or dental appointment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <f>A$1</f>
+        <v/>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Organize your health records or insurance documents.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="b">
         <v>1</v>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>A$1</f>
+        <v/>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>Add missing items to your grocery list.</t>
@@ -1674,8 +1928,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="b">
-        <v>1</v>
+      <c r="A3">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1684,8 +1939,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="b">
-        <v>1</v>
+      <c r="A4">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1694,8 +1950,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="b">
-        <v>1</v>
+      <c r="A5">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1704,8 +1961,9 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="b">
-        <v>1</v>
+      <c r="A6">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1714,8 +1972,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
-        <v>1</v>
+      <c r="A7">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1724,8 +1983,9 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
-        <v>1</v>
+      <c r="A8">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1734,8 +1994,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="b">
-        <v>1</v>
+      <c r="A9">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1744,8 +2005,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
-        <v>1</v>
+      <c r="A10">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1754,8 +2016,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
-        <v>1</v>
+      <c r="A11">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1764,8 +2027,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
-        <v>1</v>
+      <c r="A12">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1774,8 +2038,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
-        <v>1</v>
+      <c r="A13">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1784,8 +2049,9 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
-        <v>1</v>
+      <c r="A14">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1794,8 +2060,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
+      <c r="A15">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1804,8 +2071,9 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
+      <c r="A16">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1814,8 +2082,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="b">
-        <v>1</v>
+      <c r="A17">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1824,8 +2093,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="b">
-        <v>1</v>
+      <c r="A18">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1834,8 +2104,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="b">
-        <v>1</v>
+      <c r="A19">
+        <f>A$1</f>
+        <v/>
       </c>
       <c r="B19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Spreadsheet template: version identity + README stamp
Reuse the existing shared Sheet ID (onboarding page unchanged). The Apps
Script now renames the bound spreadsheet to
"MicroTasking Task Pool Template v0.1.7" and both the script and the
.xlsx builder stamp "Template version: 0.1.7 (...date...)" as README
row 2, driven by a TEMPLATE_VERSION constant kept in sync with
buildVersionBase.

README section headings are bolded by content-match (rows ending in
":") rather than hardcoded row numbers, which had drifted to the wrong
rows. Regenerated content/microtasking-sheet-template.xlsx. Updated
SPEC.md and the item 1 resume block in PUNCH_LIST.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/microtasking-sheet-template.xlsx
+++ b/content/microtasking-sheet-template.xlsx
@@ -23,13 +23,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,8 +55,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,67 +433,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MICROTASKING TASK POOL TEMPLATE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Template version: 0.1.7  (generated 2026-09-07)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Welcome to your MicroTasking Task Pool spreadsheet!</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>HOW TO USE THIS SPREADSHEET:</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1. CATEGORIES (TABS): Each tab at the bottom represents a category (e.g. Decluttering, Cleaning, Paperwork, Finances, Health, Errands).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>1. CATEGORIES (TABS): Each tab at the bottom represents a category (e.g. Decluttering, Cleaning, Paperwork, Finances, Health, Errands).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t xml:space="preserve">   - You can add new tabs, rename existing tabs, or delete tabs you don't need.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>2. COLUMNS IN TASK TABS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Column A (Row 1 Master Toggle / Checkbox): Cell A1 controls all checkboxes in Column A below it.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Check A1 to enable all tasks in the category, or uncheck A1 to disable all tasks.</t>
+          <t xml:space="preserve">   - Column A (Enabled): each task row has a checkbox. Checked = the app may suggest it; unchecked = still imported, but never suggested. Typing a description in column B adds the checkbox automatically; clearing the description removes it. Cell A1 is the master toggle for the whole tab.</t>
         </is>
       </c>
     </row>
@@ -508,7 +515,7 @@
       <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>3. SYNCING WITH THE APP:</t>
         </is>
@@ -555,24 +562,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>link</t>
+      <c r="A1" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>A$1</f>
-        <v/>
+      <c r="A2" t="b">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -581,9 +587,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <f>A$1</f>
-        <v/>
+      <c r="A3" t="b">
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -592,9 +597,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>A$1</f>
-        <v/>
+      <c r="A4" t="b">
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -603,9 +607,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>A$1</f>
-        <v/>
+      <c r="A5" t="b">
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -614,9 +617,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>A$1</f>
-        <v/>
+      <c r="A6" t="b">
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -625,9 +627,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <f>A$1</f>
-        <v/>
+      <c r="A7" t="b">
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -636,9 +637,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>A$1</f>
-        <v/>
+      <c r="A8" t="b">
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -647,9 +647,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <f>A$1</f>
-        <v/>
+      <c r="A9" t="b">
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -658,9 +657,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <f>A$1</f>
-        <v/>
+      <c r="A10" t="b">
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -669,9 +667,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <f>A$1</f>
-        <v/>
+      <c r="A11" t="b">
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -680,9 +677,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <f>A$1</f>
-        <v/>
+      <c r="A12" t="b">
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -691,9 +687,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <f>A$1</f>
-        <v/>
+      <c r="A13" t="b">
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -702,9 +697,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <f>A$1</f>
-        <v/>
+      <c r="A14" t="b">
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -713,9 +707,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <f>A$1</f>
-        <v/>
+      <c r="A15" t="b">
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -724,9 +717,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <f>A$1</f>
-        <v/>
+      <c r="A16" t="b">
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -735,9 +727,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <f>A$1</f>
-        <v/>
+      <c r="A17" t="b">
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -746,9 +737,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <f>A$1</f>
-        <v/>
+      <c r="A18" t="b">
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -757,9 +747,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <f>A$1</f>
-        <v/>
+      <c r="A19" t="b">
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -768,9 +757,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20">
-        <f>A$1</f>
-        <v/>
+      <c r="A20" t="b">
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -779,9 +767,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21">
-        <f>A$1</f>
-        <v/>
+      <c r="A21" t="b">
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -790,9 +777,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22">
-        <f>A$1</f>
-        <v/>
+      <c r="A22" t="b">
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -801,9 +787,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23">
-        <f>A$1</f>
-        <v/>
+      <c r="A23" t="b">
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -812,9 +797,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24">
-        <f>A$1</f>
-        <v/>
+      <c r="A24" t="b">
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -823,9 +807,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25">
-        <f>A$1</f>
-        <v/>
+      <c r="A25" t="b">
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -834,9 +817,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26">
-        <f>A$1</f>
-        <v/>
+      <c r="A26" t="b">
+        <v>1</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -845,9 +827,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27">
-        <f>A$1</f>
-        <v/>
+      <c r="A27" t="b">
+        <v>1</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -856,9 +837,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28">
-        <f>A$1</f>
-        <v/>
+      <c r="A28" t="b">
+        <v>1</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -867,9 +847,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29">
-        <f>A$1</f>
-        <v/>
+      <c r="A29" t="b">
+        <v>1</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -897,24 +876,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>link</t>
+      <c r="A1" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>A$1</f>
-        <v/>
+      <c r="A2" t="b">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -923,9 +901,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <f>A$1</f>
-        <v/>
+      <c r="A3" t="b">
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -934,9 +911,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>A$1</f>
-        <v/>
+      <c r="A4" t="b">
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -945,9 +921,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>A$1</f>
-        <v/>
+      <c r="A5" t="b">
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -956,9 +931,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>A$1</f>
-        <v/>
+      <c r="A6" t="b">
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -967,9 +941,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <f>A$1</f>
-        <v/>
+      <c r="A7" t="b">
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -978,9 +951,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>A$1</f>
-        <v/>
+      <c r="A8" t="b">
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -989,9 +961,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <f>A$1</f>
-        <v/>
+      <c r="A9" t="b">
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1000,9 +971,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <f>A$1</f>
-        <v/>
+      <c r="A10" t="b">
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1011,9 +981,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <f>A$1</f>
-        <v/>
+      <c r="A11" t="b">
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1022,9 +991,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <f>A$1</f>
-        <v/>
+      <c r="A12" t="b">
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1033,9 +1001,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <f>A$1</f>
-        <v/>
+      <c r="A13" t="b">
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1044,9 +1011,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <f>A$1</f>
-        <v/>
+      <c r="A14" t="b">
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1055,9 +1021,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <f>A$1</f>
-        <v/>
+      <c r="A15" t="b">
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1066,9 +1031,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <f>A$1</f>
-        <v/>
+      <c r="A16" t="b">
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1077,9 +1041,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <f>A$1</f>
-        <v/>
+      <c r="A17" t="b">
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1088,9 +1051,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <f>A$1</f>
-        <v/>
+      <c r="A18" t="b">
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1099,9 +1061,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <f>A$1</f>
-        <v/>
+      <c r="A19" t="b">
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1110,9 +1071,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20">
-        <f>A$1</f>
-        <v/>
+      <c r="A20" t="b">
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1121,9 +1081,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21">
-        <f>A$1</f>
-        <v/>
+      <c r="A21" t="b">
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1132,9 +1091,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22">
-        <f>A$1</f>
-        <v/>
+      <c r="A22" t="b">
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1143,9 +1101,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23">
-        <f>A$1</f>
-        <v/>
+      <c r="A23" t="b">
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1154,9 +1111,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24">
-        <f>A$1</f>
-        <v/>
+      <c r="A24" t="b">
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1184,24 +1140,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>link</t>
+      <c r="A1" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>A$1</f>
-        <v/>
+      <c r="A2" t="b">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1210,9 +1165,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <f>A$1</f>
-        <v/>
+      <c r="A3" t="b">
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1221,9 +1175,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>A$1</f>
-        <v/>
+      <c r="A4" t="b">
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1232,9 +1185,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>A$1</f>
-        <v/>
+      <c r="A5" t="b">
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1243,9 +1195,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>A$1</f>
-        <v/>
+      <c r="A6" t="b">
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1254,9 +1205,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <f>A$1</f>
-        <v/>
+      <c r="A7" t="b">
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1265,9 +1215,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>A$1</f>
-        <v/>
+      <c r="A8" t="b">
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1276,9 +1225,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <f>A$1</f>
-        <v/>
+      <c r="A9" t="b">
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1287,9 +1235,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <f>A$1</f>
-        <v/>
+      <c r="A10" t="b">
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1298,9 +1245,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <f>A$1</f>
-        <v/>
+      <c r="A11" t="b">
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1309,9 +1255,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <f>A$1</f>
-        <v/>
+      <c r="A12" t="b">
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1320,9 +1265,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <f>A$1</f>
-        <v/>
+      <c r="A13" t="b">
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1331,9 +1275,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <f>A$1</f>
-        <v/>
+      <c r="A14" t="b">
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1342,9 +1285,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <f>A$1</f>
-        <v/>
+      <c r="A15" t="b">
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1353,9 +1295,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <f>A$1</f>
-        <v/>
+      <c r="A16" t="b">
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1364,9 +1305,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <f>A$1</f>
-        <v/>
+      <c r="A17" t="b">
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1375,9 +1315,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <f>A$1</f>
-        <v/>
+      <c r="A18" t="b">
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1386,9 +1325,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <f>A$1</f>
-        <v/>
+      <c r="A19" t="b">
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1397,9 +1335,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20">
-        <f>A$1</f>
-        <v/>
+      <c r="A20" t="b">
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1408,9 +1345,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21">
-        <f>A$1</f>
-        <v/>
+      <c r="A21" t="b">
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1438,24 +1374,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>link</t>
+      <c r="A1" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>A$1</f>
-        <v/>
+      <c r="A2" t="b">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1464,9 +1399,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <f>A$1</f>
-        <v/>
+      <c r="A3" t="b">
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1475,9 +1409,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>A$1</f>
-        <v/>
+      <c r="A4" t="b">
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1486,9 +1419,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>A$1</f>
-        <v/>
+      <c r="A5" t="b">
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1497,9 +1429,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>A$1</f>
-        <v/>
+      <c r="A6" t="b">
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1508,9 +1439,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <f>A$1</f>
-        <v/>
+      <c r="A7" t="b">
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1519,9 +1449,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>A$1</f>
-        <v/>
+      <c r="A8" t="b">
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1530,9 +1459,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <f>A$1</f>
-        <v/>
+      <c r="A9" t="b">
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1541,9 +1469,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <f>A$1</f>
-        <v/>
+      <c r="A10" t="b">
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1552,9 +1479,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <f>A$1</f>
-        <v/>
+      <c r="A11" t="b">
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1563,9 +1489,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <f>A$1</f>
-        <v/>
+      <c r="A12" t="b">
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1574,9 +1499,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <f>A$1</f>
-        <v/>
+      <c r="A13" t="b">
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1585,9 +1509,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <f>A$1</f>
-        <v/>
+      <c r="A14" t="b">
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1596,9 +1519,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <f>A$1</f>
-        <v/>
+      <c r="A15" t="b">
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1607,9 +1529,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <f>A$1</f>
-        <v/>
+      <c r="A16" t="b">
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1618,9 +1539,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <f>A$1</f>
-        <v/>
+      <c r="A17" t="b">
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1629,9 +1549,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <f>A$1</f>
-        <v/>
+      <c r="A18" t="b">
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1640,9 +1559,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <f>A$1</f>
-        <v/>
+      <c r="A19" t="b">
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1670,24 +1588,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>link</t>
+      <c r="A1" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>A$1</f>
-        <v/>
+      <c r="A2" t="b">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1696,9 +1613,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <f>A$1</f>
-        <v/>
+      <c r="A3" t="b">
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1707,9 +1623,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>A$1</f>
-        <v/>
+      <c r="A4" t="b">
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1718,9 +1633,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>A$1</f>
-        <v/>
+      <c r="A5" t="b">
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1729,9 +1643,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>A$1</f>
-        <v/>
+      <c r="A6" t="b">
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1740,9 +1653,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <f>A$1</f>
-        <v/>
+      <c r="A7" t="b">
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1751,9 +1663,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>A$1</f>
-        <v/>
+      <c r="A8" t="b">
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1762,9 +1673,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <f>A$1</f>
-        <v/>
+      <c r="A9" t="b">
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1773,9 +1683,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <f>A$1</f>
-        <v/>
+      <c r="A10" t="b">
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1784,9 +1693,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <f>A$1</f>
-        <v/>
+      <c r="A11" t="b">
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1795,9 +1703,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <f>A$1</f>
-        <v/>
+      <c r="A12" t="b">
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1806,9 +1713,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <f>A$1</f>
-        <v/>
+      <c r="A13" t="b">
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1817,9 +1723,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <f>A$1</f>
-        <v/>
+      <c r="A14" t="b">
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1828,9 +1733,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <f>A$1</f>
-        <v/>
+      <c r="A15" t="b">
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1839,9 +1743,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <f>A$1</f>
-        <v/>
+      <c r="A16" t="b">
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1850,9 +1753,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <f>A$1</f>
-        <v/>
+      <c r="A17" t="b">
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1861,9 +1763,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <f>A$1</f>
-        <v/>
+      <c r="A18" t="b">
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1872,9 +1773,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <f>A$1</f>
-        <v/>
+      <c r="A19" t="b">
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1902,24 +1802,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>link</t>
+      <c r="A1" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>A$1</f>
-        <v/>
+      <c r="A2" t="b">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1928,9 +1827,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <f>A$1</f>
-        <v/>
+      <c r="A3" t="b">
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1939,9 +1837,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>A$1</f>
-        <v/>
+      <c r="A4" t="b">
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1950,9 +1847,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>A$1</f>
-        <v/>
+      <c r="A5" t="b">
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1961,9 +1857,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>A$1</f>
-        <v/>
+      <c r="A6" t="b">
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1972,9 +1867,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <f>A$1</f>
-        <v/>
+      <c r="A7" t="b">
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1983,9 +1877,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>A$1</f>
-        <v/>
+      <c r="A8" t="b">
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1994,9 +1887,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <f>A$1</f>
-        <v/>
+      <c r="A9" t="b">
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -2005,9 +1897,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <f>A$1</f>
-        <v/>
+      <c r="A10" t="b">
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -2016,9 +1907,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <f>A$1</f>
-        <v/>
+      <c r="A11" t="b">
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -2027,9 +1917,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <f>A$1</f>
-        <v/>
+      <c r="A12" t="b">
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -2038,9 +1927,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <f>A$1</f>
-        <v/>
+      <c r="A13" t="b">
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2049,9 +1937,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <f>A$1</f>
-        <v/>
+      <c r="A14" t="b">
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2060,9 +1947,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <f>A$1</f>
-        <v/>
+      <c r="A15" t="b">
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2071,9 +1957,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <f>A$1</f>
-        <v/>
+      <c r="A16" t="b">
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -2082,9 +1967,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <f>A$1</f>
-        <v/>
+      <c r="A17" t="b">
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -2093,9 +1977,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <f>A$1</f>
-        <v/>
+      <c r="A18" t="b">
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -2104,9 +1987,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <f>A$1</f>
-        <v/>
+      <c r="A19" t="b">
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
README tab: readability + tab-order / task-order notes
- Column A: fixed width (700px / xlsx 95) + wrap, instead of
  autoResizeColumn blowing the column out to the longest sentence.
- Split "1. CATEGORIES (TABS):" onto its own bold line; blank line
  under "HOW TO USE THIS SPREADSHEET:".
- New content: tab order drives category weighting (leftmost enabled
  ~2x the rightmost, linear between - matches chooseWeightedTask), and
  a note that task-row order within a tab doesn't affect the odds.

README text lives in both populate_google_sheet.js and
generate_sheet_template.py; kept in sync. xlsx regenerated, script
pushed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/microtasking-sheet-template.xlsx
+++ b/content/microtasking-sheet-template.xlsx
@@ -55,9 +55,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -426,10 +431,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,17 +452,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Welcome to your MicroTasking Task Pool spreadsheet!</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -467,76 +472,100 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1. CATEGORIES (TABS): Each tab at the bottom represents a category (e.g. Decluttering, Cleaning, Paperwork, Finances, Health, Errands).</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - You can add new tabs, rename existing tabs, or delete tabs you don't need.</t>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>1. CATEGORIES (TABS):</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Each tab at the bottom is a category (e.g. Decluttering, Cleaning, Paperwork, Finances, Health, Errands).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - You can add, rename, delete, and rearrange tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Tab order sets the odds: tasks in your leftmost enabled category are about twice as likely to be assigned as tasks in your rightmost enabled category, sliding linearly in between. Enable or disable categories in the app's settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>2. COLUMNS IN TASK TABS:</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Column A (Enabled): each task row has a checkbox. Checked = the app may suggest it; unchecked = still imported, but never suggested. Typing a description in column B adds the checkbox automatically; clearing a row's description deletes the whole row. Cell A1 is the master toggle for the whole tab.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Column B (Description): The text description of the micro-task.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Column C (Link): Optional URL (e.g. video tutorial, document, or web tool).</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - The order of task rows within a tab does not affect how often a task is assigned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>3. SYNCING WITH THE APP:</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Set Share permissions to 'Anyone with the link can view'.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Paste your Sheet URL into the onboarding page to generate your custom QR code.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   - In the MicroTasking app, tap Settings -&gt; Import External Task Pool -&gt; Scan QR Code.</t>
         </is>
@@ -562,15 +591,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -876,15 +905,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1140,15 +1169,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1374,15 +1403,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1588,15 +1617,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1802,15 +1831,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>

</xml_diff>